<commit_message>
data: update review_products.xlsx with first batch of 5 office products
</commit_message>
<xml_diff>
--- a/review_products.xlsx
+++ b/review_products.xlsx
@@ -472,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -521,41 +521,10 @@
       </c>
     </row>
     <row r="2" ht="39.95" customHeight="1">
-      <c r="A2" s="2" t="n">
+      <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>วางรายละเอียดสินค้าจาก Shopee ทั้งหมดที่นี่</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.shopee.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>https://s.lazada.co.th/xxx</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>https://down-th.img.susercontent.com/xxx.jpg</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>ลด 20%</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="345" customHeight="1">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>RAY-BAN JUSTIN- RB4165F 601/71
 Ray-Ban เรแบนเป็นผู้นำด้านการผลิตแว่นกันแดด และแว่นสายตา ที่ได้ความนิยมมากที่สุดทั่วโลก มีให้เลือกหลากหลายสไตล์ เหมาะกับทุกคน และใส่ได้ทั้งผู้หญิงและผู้ชาย
@@ -569,23 +538,23 @@
 Lens Material: Polycarbonate Standard</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/AUqz80oxUd</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6PzJE?c=b&amp;t=p-ijr1Q-svKWG</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134201-7r990-lscec08f21gm73.webp
 https://down-th.img.susercontent.com/file/th-11134201-7r98y-lscec0amysmu78.webp</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿5,130
 final price indicator icon
@@ -597,17 +566,17 @@
 </t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>done 2026-05-21 13:15</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409.5" customHeight="1">
-      <c r="A4" t="n">
+    <row r="3" ht="345" customHeight="1">
+      <c r="A3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>Sony BRAVIA 3 ทีวี 55 นิ้ว รุ่น K-55S30 4K Ultra HD Smart TV (Google TV) | 4K HDR Processor X1
 รายละเอียดสินค้า
@@ -627,22 +596,22 @@
 เรียกดูภาพยนตร์และรายการทีวีมากกว่า 400,000 ตอนจากบริการสตรีมมิ่งของคุณทั้งหมดในที่เดียว โดยจัดเป็นหัวข้อและแนวเนื้อหาไว้ตามสิ่งที่คุณสนใจ</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t>https://s.shopee.co.th/10zvLKc6Ji</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://s.lazada.co.th/s.Z6mEyG?c=a&amp;t=p-i0-s0&amp;sub_id1=W1</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>https://down-th.img.susercontent.com/file/th-11134207-7r98v-lvsn9yh5vql9c5.webp</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F3" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">฿20,500
 final price indicator icon
@@ -650,6 +619,136 @@
 โค้ดส่วนลดร้านค้า
 ลด ฿1.99k
 </t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409.5" customHeight="1">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>เบาะพกพา เบาะสุขภาพ เบาะเก้าอี้ เบาะรองเอว นั่งนานไม่เมื่อย เบาะรองนั่งเพื่อสุขภาพ เก้าอี้รองปรับท่านั่ง หมอนรองหลัง</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/2LVQzcZ3Ip</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-7qul7-lgesv2vzlg0ec1.webp</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ลด 69% เหลือ ฿499 (ปกติ ฿1,599)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>(พร้อมส่งจากไทย) เบาะรองนั่ง พร้อมพิงหลัง หูการ์ตุน มีสายรัดเก้าอี้ เบาะรองหลัง</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6L1Zl7G3F4</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-7r98z-ln4pqmcm29mxa6.webp</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ลด 5% เริ่มต้น ฿160 - ฿199</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ไฟฟ้า High-End เก้าอี้สํานักงานหนังแท้ Boss เก้าอี้ขนาดใหญ่ Ergonomic เก้าอี้ Reclining Liftable นวดบ้านการเรียนรู้เก้าอี้คอมพิวเตอร์</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8piujnmmou</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/sg-11134201-824j0-mdzysm91y1a830.webp</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ลด 50% เริ่มต้น ฿14,534 - ฿43,359</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>[ลดอาการปวดข้อมือ] แผ่นรองเมาส์/ที่รองข้อมือ/เมมโมรี่โฟม/แผ่นรองคีย์บอร์ด</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/70HGYal3GC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/sg-11134201-825zp-mkjcbxcbzz7s79.webp</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ลด 49% เริ่มต้น ฿163 - ฿183</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Screenbar Light Bar โคมไฟแขวนจอคอม LED ปรับไฟได้ 3 สี ปรับองศาได้หลายมุม ลดแสงสีฟ้า</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/6VKzxnaa2h</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-7r98p-lvcxws3wijsqf6.webp</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ลด 46% เริ่มต้น ฿269 - ฿700</t>
         </is>
       </c>
     </row>

</xml_diff>